<commit_message>
refactor: localization & luban
</commit_message>
<xml_diff>
--- a/Config/Excels/Tables/Audio_audio.xlsx
+++ b/Config/Excels/Tables/Audio_audio.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="16665" windowHeight="7650"/>
+    <workbookView windowWidth="27945" windowHeight="12375"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>##var</t>
   </si>
@@ -66,9 +66,6 @@
     <t>volume</t>
   </si>
   <si>
-    <t>inPool</t>
-  </si>
-  <si>
     <t>##</t>
   </si>
   <si>
@@ -87,29 +84,10 @@
     <t>##group</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF006100"/>
-        <rFont val="等线"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>这是i</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF006100"/>
-        <rFont val="等线"/>
-        <charset val="134"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>d</t>
-    </r>
-  </si>
-  <si>
-    <t>音频类型(0声音音效、1UI音效、2背景音乐、3人声神效、4最大声效)</t>
+    <t>自增Id</t>
+  </si>
+  <si>
+    <t>音频类型 0-Sound 1-UISound 2-Music 3-Voice 4-Ambient</t>
   </si>
   <si>
     <t>音乐名称</t>
@@ -119,9 +97,6 @@
   </si>
   <si>
     <t>音量(0-100)</t>
-  </si>
-  <si>
-    <t>池化(对于贯穿游戏流程较长的音频需要存到资源池)</t>
   </si>
   <si>
     <t>备注</t>
@@ -1082,7 +1057,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:AB6"/>
+  <dimension ref="A1:AA6"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.25" outlineLevelRow="5"/>
   <cols>
     <col min="1" max="1" width="13.125" customWidth="1"/>
@@ -1091,11 +1066,10 @@
     <col min="4" max="4" width="30" customWidth="1"/>
     <col min="5" max="5" width="12.25" customWidth="1"/>
     <col min="6" max="6" width="18.75" customWidth="1"/>
-    <col min="7" max="7" width="41.75" customWidth="1"/>
-    <col min="8" max="8" width="24.75" customWidth="1"/>
+    <col min="7" max="7" width="24.75" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" spans="1:28">
+    <row r="1" s="1" customFormat="1" spans="1:27">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1117,9 +1091,7 @@
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
-        <v>7</v>
-      </c>
+      <c r="H1"/>
       <c r="I1"/>
       <c r="J1"/>
       <c r="K1"/>
@@ -1139,9 +1111,8 @@
       <c r="Y1"/>
       <c r="Z1"/>
       <c r="AA1"/>
-      <c r="AB1"/>
     </row>
-    <row r="2" s="1" customFormat="1" spans="1:28">
+    <row r="2" s="1" customFormat="1" spans="1:27">
       <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
@@ -1151,7 +1122,7 @@
       <c r="E2" s="3"/>
       <c r="F2" s="3"/>
       <c r="G2" s="3"/>
-      <c r="H2" s="3"/>
+      <c r="H2"/>
       <c r="I2"/>
       <c r="J2"/>
       <c r="K2"/>
@@ -1171,33 +1142,30 @@
       <c r="Y2"/>
       <c r="Z2"/>
       <c r="AA2"/>
-      <c r="AB2"/>
     </row>
-    <row r="3" s="2" customFormat="1" spans="1:28">
+    <row r="3" s="2" customFormat="1" spans="1:27">
       <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C3" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="E3" s="4" t="s">
-        <v>11</v>
-      </c>
       <c r="F3" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>7</v>
-      </c>
+        <v>6</v>
+      </c>
+      <c r="H3"/>
       <c r="I3"/>
       <c r="J3"/>
       <c r="K3"/>
@@ -1217,11 +1185,10 @@
       <c r="Y3"/>
       <c r="Z3"/>
       <c r="AA3"/>
-      <c r="AB3"/>
     </row>
-    <row r="4" s="2" customFormat="1" spans="1:28">
+    <row r="4" s="2" customFormat="1" spans="1:27">
       <c r="A4" s="4" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -1229,7 +1196,7 @@
       <c r="E4" s="4"/>
       <c r="F4" s="4"/>
       <c r="G4" s="4"/>
-      <c r="H4" s="4"/>
+      <c r="H4"/>
       <c r="I4"/>
       <c r="J4"/>
       <c r="K4"/>
@@ -1249,33 +1216,30 @@
       <c r="Y4"/>
       <c r="Z4"/>
       <c r="AA4"/>
-      <c r="AB4"/>
     </row>
-    <row r="5" s="1" customFormat="1" spans="1:28">
+    <row r="5" s="1" customFormat="1" spans="1:27">
       <c r="A5" s="3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="D5" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="E5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="3" t="s">
+      <c r="F5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="G5" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="G5" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5" s="3" t="s">
-        <v>19</v>
-      </c>
+      <c r="H5"/>
       <c r="I5"/>
       <c r="J5"/>
       <c r="K5"/>
@@ -1295,9 +1259,8 @@
       <c r="Y5"/>
       <c r="Z5"/>
       <c r="AA5"/>
-      <c r="AB5"/>
     </row>
-    <row r="6" spans="2:8">
+    <row r="6" spans="1:27">
       <c r="B6">
         <v>10001</v>
       </c>
@@ -1313,11 +1276,8 @@
       <c r="F6">
         <v>60</v>
       </c>
-      <c r="G6" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H6" s="5" t="s">
-        <v>20</v>
+      <c r="G6" s="5" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>